<commit_message>
DRIV-1606 | replaced template files with the new provided by zafar
</commit_message>
<xml_diff>
--- a/public/ApplicantsTemplate.xlsx
+++ b/public/ApplicantsTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10611"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/julia4/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MM-HO HP New\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C50C295-D9EB-A940-A5B2-88B8906280F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{542FEC91-7B72-4C08-BA0B-A28617F4C067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="20740" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Import Applicants Template" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="64">
   <si>
     <t>first_name</t>
   </si>
@@ -161,9 +161,6 @@
   </si>
   <si>
     <t>assignedUserId</t>
-  </si>
-  <si>
-    <t>is_hired</t>
   </si>
   <si>
     <t>remarks</t>
@@ -725,57 +722,56 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:AR9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:AQ9"/>
+  <sheetFormatPr defaultColWidth="10.5" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.375" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.375" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.625" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.875" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.625" style="1" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="20" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.875" style="1" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="17.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="22.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="24.1640625" style="20" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="27.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="8.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="23.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="14.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="20.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="12.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="23.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="13.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="22.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="24.125" style="20" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="27.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="8.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="23.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="13.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="14.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="14.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="20.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="12.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="23.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="15.625" style="1" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="21.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="23.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="16.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="22.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="19.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="23.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="16.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="22.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="19.625" style="1" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="13.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="7.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="33" style="1" bestFit="1" customWidth="1"/>
-    <col min="44" max="1018" width="10.5" style="1"/>
-    <col min="1019" max="1024" width="8.33203125" style="1" customWidth="1"/>
-    <col min="1025" max="16384" width="10.5" style="1"/>
+    <col min="42" max="42" width="33" style="1" bestFit="1" customWidth="1"/>
+    <col min="43" max="1017" width="10.5" style="1"/>
+    <col min="1018" max="1023" width="8.375" style="1" customWidth="1"/>
+    <col min="1024" max="16384" width="10.5" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -905,58 +901,55 @@
       <c r="AQ1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" s="1" t="s">
-        <v>43</v>
-      </c>
     </row>
-    <row r="2" spans="1:44" s="12" customFormat="1" ht="34" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:43" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E2" s="15">
         <v>30043</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I2" s="12">
         <v>54466</v>
       </c>
       <c r="J2" s="12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K2" s="16">
         <v>47239</v>
       </c>
       <c r="L2" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="M2" s="12" t="s">
         <v>45</v>
-      </c>
-      <c r="M2" s="12" t="s">
-        <v>46</v>
       </c>
       <c r="N2" s="12">
         <v>10</v>
       </c>
       <c r="O2" s="12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="P2" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="Q2" s="17" t="b">
         <f>TRUE()</f>
@@ -967,26 +960,26 @@
         <v>0</v>
       </c>
       <c r="S2" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="T2" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="T2" s="12" t="s">
+      <c r="U2" s="12" t="s">
         <v>49</v>
-      </c>
-      <c r="U2" s="12" t="s">
-        <v>50</v>
       </c>
       <c r="V2" s="17" t="b">
         <f>TRUE()</f>
         <v>1</v>
       </c>
       <c r="W2" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="X2" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="Y2" s="12" t="s">
         <v>51</v>
-      </c>
-      <c r="X2" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="Y2" s="12" t="s">
-        <v>52</v>
       </c>
       <c r="Z2" s="17" t="b">
         <f>TRUE()</f>
@@ -996,7 +989,7 @@
         <v>3</v>
       </c>
       <c r="AB2" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AC2" s="12">
         <v>0</v>
@@ -1006,14 +999,14 @@
         <v>0</v>
       </c>
       <c r="AF2" s="12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="AG2" s="17" t="b">
         <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="AH2" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AI2" s="17" t="b">
         <f>FALSE()</f>
@@ -1023,42 +1016,38 @@
         <v>0</v>
       </c>
       <c r="AK2" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AL2" s="17" t="b">
         <f>FALSE()</f>
         <v>0</v>
       </c>
       <c r="AM2" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="AN2" s="12" t="s">
         <v>54</v>
-      </c>
-      <c r="AN2" s="12" t="s">
-        <v>55</v>
       </c>
       <c r="AO2" s="12">
         <v>2</v>
       </c>
-      <c r="AP2" s="17" t="b">
-        <f>FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="AQ2" s="18" t="s">
+      <c r="AP2" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="AQ2" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="AR2" s="12" t="s">
-        <v>57</v>
-      </c>
     </row>
-    <row r="3" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:43" x14ac:dyDescent="0.25">
       <c r="C3" s="4"/>
       <c r="F3" s="12"/>
     </row>
-    <row r="4" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:43" x14ac:dyDescent="0.25">
       <c r="C4" s="4"/>
       <c r="D4" s="7"/>
       <c r="I4" s="11"/>
     </row>
-    <row r="5" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:43" x14ac:dyDescent="0.25">
       <c r="C5" s="4"/>
       <c r="D5" s="2"/>
       <c r="E5" s="10"/>
@@ -1066,20 +1055,20 @@
       <c r="J5" s="22"/>
       <c r="K5" s="8"/>
     </row>
-    <row r="6" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:43" x14ac:dyDescent="0.25">
       <c r="D6" s="7"/>
       <c r="I6" s="11"/>
     </row>
-    <row r="7" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:43" x14ac:dyDescent="0.25">
       <c r="I7" s="11"/>
       <c r="J7" s="23"/>
     </row>
-    <row r="8" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:43" x14ac:dyDescent="0.25">
       <c r="I8" s="11"/>
       <c r="K8" s="8"/>
       <c r="X8" s="21"/>
     </row>
-    <row r="9" spans="1:44" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:43" x14ac:dyDescent="0.25">
       <c r="C9" s="9"/>
       <c r="D9" s="7"/>
       <c r="K9" s="8"/>
@@ -1121,11 +1110,11 @@
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Notify final remarks of applicant" sqref="AQ1:AQ1003" xr:uid="{52C29A08-857B-4FCA-ADBE-1E01E6063021}">
+    <dataValidation operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Notify final remarks of applicant" sqref="AP1:AP1003" xr:uid="{52C29A08-857B-4FCA-ADBE-1E01E6063021}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Some extra notes for applicant " sqref="AR1:AR1003" xr:uid="{E1B8C449-D439-4BF6-A0CC-EB60A2D01F73}">
+    <dataValidation operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Some extra notes for applicant " sqref="AQ1:AQ1003" xr:uid="{E1B8C449-D439-4BF6-A0CC-EB60A2D01F73}">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1152,7 +1141,7 @@
       <formula1>0</formula1>
       <formula2>1111</formula2>
     </dataValidation>
-    <dataValidation operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Preffered Location" prompt="You can select multiple options from the following_x000a_LOCAL_x000a_OTR_x000a_REGIONAL" sqref="O1:O1048576" xr:uid="{0392F7BC-B7D0-4B18-BB93-C14CC9E2751E}"/>
+    <dataValidation operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Preferred Location" prompt="You can add multiple options from the following;_x000a_LOCAL_x000a_OTR_x000a_REGIONAL" sqref="O1:O1048576" xr:uid="{0392F7BC-B7D0-4B18-BB93-C14CC9E2751E}"/>
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Input" error="Please enter valid ID" promptTitle="Assigned User" prompt="ID of user to whome you want to assign this applicant" sqref="AO1:AO1048576" xr:uid="{9F201353-8F5E-4451-AE4E-B6645CF6BDA6}">
       <formula1>0</formula1>
       <formula2>10000</formula2>
@@ -1193,7 +1182,7 @@
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Entry" error="Please enter a valid value: TRUE or FALSE." promptTitle="Accepted Values" prompt="Please select one of the following values: TRUE, FALSE." sqref="AP1:AP1048576 AL1:AL1048576" xr:uid="{095163CC-AEA2-4C88-A2FB-77B8F566E04A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Entry" error="Please enter a valid value: TRUE or FALSE." promptTitle="Accepted Values" prompt="Please select one of the following values: TRUE, FALSE." sqref="AL1:AL1048576" xr:uid="{095163CC-AEA2-4C88-A2FB-77B8F566E04A}">
       <formula1>"TRUE, FALSE"</formula1>
     </dataValidation>
     <dataValidation type="list" operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Entry" error="Please enter a valid value: TRUE or FALSE." promptTitle="Accepted Values" prompt="Please select one of the following values: TRUE, FALSE." sqref="AI1:AI1048576 AE1:AE1048576 Z1:Z1048576 V1:V1048576 R1:R1048576" xr:uid="{CE6216D9-CDF5-4EE0-9DDF-7D95450CD32C}">
@@ -1202,9 +1191,7 @@
     <dataValidation type="list" operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Entry" error="Please enter a valid value: TRUE or FALSE." prompt="Please select one of the following values: TRUE, FALSE." sqref="AG1:AG1048576" xr:uid="{EE251DFC-E7C0-47A0-9582-488538272061}">
       <formula1>"TRUE, FALSE"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Select Endorsement" prompt="Please select endorsement from the following;_x000a_HAZMAT_x000a_TANKERS_x000a_DOUBLES_TRIPLES_x000a_SCHOOL_BUS_x000a_TWIC_x000a__x000a_Note : Input is Case Sensitive." sqref="T1:T1048576" xr:uid="{8E4834E0-EE55-4DD7-964E-6ED50A34B8DF}">
-      <formula1>"HAZMAT,TANKERS,DOUBLES_TRIPLES,SCHOOL_BUS,TWIC"</formula1>
-    </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Endorsements/TWIC" prompt="Please add endorsements and qualifications you have:_x000a_HAZMAT_x000a_TANKERS_x000a_DOUBLES_TRIPLES_x000a_SCHOOL_BUS_x000a_TWIC_x000a__x000a_Note : Input is Case Sensitive." sqref="T1:T1048576" xr:uid="{8E4834E0-EE55-4DD7-964E-6ED50A34B8DF}"/>
     <dataValidation type="list" operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Entry" error="Please enter a valid value: TRUE " promptTitle="Accepted Values" prompt="This must be TRUE" sqref="Q1:Q1048576" xr:uid="{AB0E5FE3-0748-475D-849D-5F9A89EDD97E}">
       <formula1>"TRUE"</formula1>
     </dataValidation>
@@ -1214,9 +1201,7 @@
     <dataValidation type="list" operator="equal" showInputMessage="1" showErrorMessage="1" errorTitle="Highest Degree" error="Please put proper value" promptTitle="The valid highest degress values are the following:" prompt="HIGH_SCHOOL_x000a_ASSOCIATE_x000a_BACHELOR_x000a_MASTER_x000a_DOCTORAL_x000a__x000a_Note : Input is Case Sensitive." sqref="U1:U1048576" xr:uid="{259DA3E7-19A6-49F7-906A-7AEA601F56FA}">
       <formula1>"HIGH_SCHOOL,ASSOCIATE,BACHELOR,MASTER,DOCTORAL"</formula1>
     </dataValidation>
-    <dataValidation type="list" operator="equal" showInputMessage="1" showErrorMessage="1" errorTitle="Transmission Type" error="Please add proper value" promptTitle="The accepted transmission types are as follows" prompt="MANUAL_x000a_AUTOMATIC_x000a__x000a_Note : Input is Case Sensitive." sqref="S1:S1048576" xr:uid="{158793F1-647D-4C1C-A937-4B9E37F8A6D0}">
-      <formula1>"MANUAL,AUTOMATIC"</formula1>
-    </dataValidation>
+    <dataValidation operator="equal" showInputMessage="1" showErrorMessage="1" errorTitle="Transmission Type" error="Please add proper value" promptTitle="The accepted transmission types are as follows" prompt="MANUAL_x000a_AUTOMATIC_x000a__x000a_Note : Input is Case Sensitive." sqref="S1:S1048576" xr:uid="{158793F1-647D-4C1C-A937-4B9E37F8A6D0}"/>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{F2F26B8D-DCEC-4F28-B3BD-6F952843A6A7}"/>

</xml_diff>